<commit_message>
UPDATE COM VERSÃO DESKTOP
</commit_message>
<xml_diff>
--- a/src/output/pop_final.xlsx
+++ b/src/output/pop_final.xlsx
@@ -472,11 +472,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>[31, 26, 31, 31, 19]</t>
+          <t>[24, 18, 18, 24, 18]</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>40.49047096288861</v>
+        <v>50.63540522778678</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -484,7 +484,7 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>138</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3">
@@ -499,15 +499,15 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>[26, 13, 16, 25, 11]</t>
+          <t>[15, 25, 11, 27, 28]</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>102.8162559677071</v>
+        <v>110.9099566504517</v>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>91</v>
+        <v>106</v>
       </c>
     </row>
     <row r="4">
@@ -522,15 +522,15 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>[12, 24, 30, 8, 0]</t>
+          <t>[19, 24, 16, 3, 4]</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>81.64049932078191</v>
+        <v>105.5993524413959</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>74</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5">
@@ -545,15 +545,15 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>[18, 20, 7, 21, 22]</t>
+          <t>[13, 25, 5, 0, 2]</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>137.3376955045644</v>
+        <v>84.35566571140188</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
-        <v>88</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6">
@@ -568,15 +568,15 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>[6, 26, 18, 17, 16]</t>
+          <t>[10, 27, 7, 30, 22]</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>121.1844124694973</v>
+        <v>92.25317926118218</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
-        <v>83</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>